<commit_message>
Added Claude-generated script to add option to look at strain (q/q0) in Andrew's viewer
</commit_message>
<xml_diff>
--- a/test_calcs.xlsx
+++ b/test_calcs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mines0-my.sharepoint.com/personal/benschne_mines_edu/Documents/Code/Python/Analysis_pyFAI-1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="8_{C7C7E276-6A03-F043-BD40-304A7890F963}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37612356-E9D2-E044-851B-D31022639BA0}"/>
+  <xr:revisionPtr revIDLastSave="63" documentId="8_{C7C7E276-6A03-F043-BD40-304A7890F963}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7C259DFD-594A-EE4C-8D50-55CD4660C248}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="160" yWindow="760" windowWidth="29920" windowHeight="17480" xr2:uid="{77C8FE66-F471-6F4F-880B-A0D9347144D5}"/>
+    <workbookView xWindow="160" yWindow="760" windowWidth="29920" windowHeight="17480" xr2:uid="{77C8FE66-F471-6F4F-880B-A0D9347144D5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -144,6 +144,36 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="2400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Fityk</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> Fits Plot (Bkg Subtracted, No Filtering of Fits)</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -157,7 +187,7 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+            <a:defRPr sz="2400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="65000"/>
@@ -175,7 +205,17 @@
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.13903127924467168"/>
+          <c:y val="7.2359236053783735E-2"/>
+          <c:w val="0.83916816019678064"/>
+          <c:h val="0.75730181564393984"/>
+        </c:manualLayout>
+      </c:layout>
       <c:scatterChart>
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
@@ -6379,6 +6419,61 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Azimuth (º)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -6387,10 +6482,7 @@
           <a:noFill/>
           <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
+              <a:schemeClr val="tx1"/>
             </a:solidFill>
             <a:round/>
           </a:ln>
@@ -6401,7 +6493,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -6417,7 +6509,7 @@
           </a:p>
         </c:txPr>
         <c:crossAx val="1301941599"/>
-        <c:crosses val="autoZero"/>
+        <c:crossesAt val="-2.5000000000000005E-3"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
@@ -6441,6 +6533,61 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>ln(Frame 492 / Frame  304)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -6449,10 +6596,7 @@
           <a:noFill/>
           <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
+              <a:schemeClr val="tx1"/>
             </a:solidFill>
             <a:round/>
           </a:ln>
@@ -6463,7 +6607,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -6479,19 +6623,31 @@
           </a:p>
         </c:txPr>
         <c:crossAx val="1016069728"/>
-        <c:crosses val="autoZero"/>
+        <c:crossesAt val="-2.5000000000000005E-3"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
-        <a:ln>
-          <a:noFill/>
+        <a:ln w="19050">
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
         </a:ln>
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.14166591575235257"/>
+          <c:y val="0.72621741292404263"/>
+          <c:w val="0.7514126723087764"/>
+          <c:h val="5.4934261365444756E-2"/>
+        </c:manualLayout>
+      </c:layout>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -6505,7 +6661,7 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+            <a:defRPr sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="65000"/>
@@ -6552,7 +6708,7 @@
     <a:lstStyle/>
     <a:p>
       <a:pPr>
-        <a:defRPr/>
+        <a:defRPr sz="2000"/>
       </a:pPr>
       <a:endParaRPr lang="en-US"/>
     </a:p>
@@ -7125,16 +7281,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>22310</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>112927</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>382715</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>188784</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>33</xdr:col>
-      <xdr:colOff>617838</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>34324</xdr:rowOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>669324</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>154460</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>

</xml_diff>